<commit_message>
Label section references in catalogue content sheets
</commit_message>
<xml_diff>
--- a/Тематика для рассылки/Готовые файлы/01_Анкета_преподавателя_Rozum.xlsx
+++ b/Тематика для рассылки/Готовые файлы/01_Анкета_преподавателя_Rozum.xlsx
@@ -7723,7 +7723,7 @@
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 60</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 60</t>
         </is>
       </c>
       <c r="B9" s="4" t="n"/>
@@ -7820,7 +7820,7 @@
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 14</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B18" s="4" t="n"/>
@@ -7917,7 +7917,7 @@
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 16</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B27" s="4" t="n"/>
@@ -8014,7 +8014,7 @@
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 15</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B36" s="4" t="n"/>
@@ -8111,7 +8111,7 @@
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 25</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B45" s="4" t="n"/>
@@ -8208,7 +8208,7 @@
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сбор данных и предотвращение атак · УТП: таблица 2, строка 18</t>
+Раздел: Сбор данных и предотвращение атак · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B54" s="4" t="n"/>
@@ -8305,7 +8305,7 @@
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 28</t>
+Раздел: Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 28</t>
         </is>
       </c>
       <c r="B63" s="4" t="n"/>
@@ -8402,7 +8402,7 @@
       <c r="A72" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сбор данных и предотвращение атак · УТП: таблица 2, строка 19</t>
+Раздел: Сбор данных и предотвращение атак · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B72" s="4" t="n"/>
@@ -8499,7 +8499,7 @@
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Нулевая бюрократия и клиентоцентричность · УТП: таблица 2, строка 14</t>
+Раздел: Нулевая бюрократия и клиентоцентричность · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B81" s="4" t="n"/>
@@ -8648,7 +8648,7 @@
       <c r="A94" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 23</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B94" s="4" t="n"/>
@@ -8745,7 +8745,7 @@
       <c r="A103" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 10</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B103" s="4" t="n"/>
@@ -8842,7 +8842,7 @@
       <c r="A112" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 23</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B112" s="4" t="n"/>
@@ -8939,7 +8939,7 @@
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 24</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 24</t>
         </is>
       </c>
       <c r="B121" s="4" t="n"/>
@@ -9036,7 +9036,7 @@
       <c r="A130" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 23</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B130" s="4" t="n"/>
@@ -9185,7 +9185,7 @@
       <c r="A143" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 18</t>
+Раздел: Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B143" s="4" t="n"/>
@@ -9282,7 +9282,7 @@
       <c r="A152" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 22</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B152" s="4" t="n"/>
@@ -9392,7 +9392,7 @@
       <c r="A162" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 29</t>
+Раздел: Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 29</t>
         </is>
       </c>
       <c r="B162" s="4" t="n"/>
@@ -9489,7 +9489,7 @@
       <c r="A171" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Связь SOAR/TI/SIEM · УТП: таблица 2, строка 69</t>
+Раздел: Связь SOAR/TI/SIEM · УТП: таблица 2, строка 69</t>
         </is>
       </c>
       <c r="B171" s="4" t="n"/>
@@ -9781,7 +9781,7 @@
       <c r="A195" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Основы функционирования информационных систем · УТП: таблица 2, строка 9</t>
+Раздел: Основы функционирования информационных систем · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B195" s="4" t="n"/>
@@ -9956,7 +9956,7 @@
       <c r="A210" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 22</t>
+Раздел: Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B210" s="4" t="n"/>
@@ -10053,7 +10053,7 @@
       <c r="A219" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B219" s="4" t="n"/>
@@ -10131,7 +10131,7 @@
       <c r="A225" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 12</t>
+Раздел: Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B225" s="4" t="n"/>
@@ -10228,7 +10228,7 @@
       <c r="A234" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 22</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B234" s="4" t="n"/>
@@ -10377,7 +10377,7 @@
       <c r="A247" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Методологические основы обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 11</t>
+Раздел: Методологические основы обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B247" s="4" t="n"/>
@@ -10539,7 +10539,7 @@
       <c r="A261" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B261" s="4" t="n"/>
@@ -10636,7 +10636,7 @@
       <c r="A270" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B270" s="4" t="n"/>
@@ -10824,7 +10824,7 @@
       <c r="A286" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 16</t>
+Раздел: Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B286" s="4" t="n"/>
@@ -10921,7 +10921,7 @@
       <c r="A295" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Управление доступом и аутентификация · УТП: таблица 2, строка 24</t>
+Раздел: Управление доступом и аутентификация · УТП: таблица 2, строка 24</t>
         </is>
       </c>
       <c r="B295" s="4" t="n"/>
@@ -11018,7 +11018,7 @@
       <c r="A304" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 46</t>
+Раздел: Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 46</t>
         </is>
       </c>
       <c r="B304" s="4" t="n"/>
@@ -11141,7 +11141,7 @@
       <c r="A315" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 22</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B315" s="4" t="n"/>
@@ -11316,7 +11316,7 @@
       <c r="A330" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Применение ИИ в ИБ · УТП: таблица 2, строка 16</t>
+Раздел: Применение ИИ в ИБ · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B330" s="4" t="n"/>
@@ -11439,7 +11439,7 @@
       <c r="A341" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 20</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B341" s="4" t="n"/>
@@ -11536,7 +11536,7 @@
       <c r="A350" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 20</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B350" s="4" t="n"/>
@@ -11633,7 +11633,7 @@
       <c r="A359" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 21</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B359" s="4" t="n"/>
@@ -11698,7 +11698,7 @@
       <c r="A364" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Методологические основы обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 11</t>
+Раздел: Методологические основы обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B364" s="4" t="n"/>
@@ -11834,7 +11834,7 @@
       <c r="A376" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 21</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B376" s="4" t="n"/>
@@ -11964,7 +11964,7 @@
       <c r="A386" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 19</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B386" s="4" t="n"/>
@@ -12113,7 +12113,7 @@
       <c r="A399" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Основы ИИ и машинного обучения · УТП: таблица 2, строка 6</t>
+Раздел: Основы ИИ и машинного обучения · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B399" s="4" t="n"/>
@@ -12210,7 +12210,7 @@
       <c r="A408" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Основы криптографической защиты информации · УТП: таблица 2, строка 6</t>
+Раздел: Основы криптографической защиты информации · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B408" s="4" t="n"/>
@@ -12307,7 +12307,7 @@
       <c r="A417" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 13</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B417" s="4" t="n"/>
@@ -12404,7 +12404,7 @@
       <c r="A426" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 19</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B426" s="4" t="n"/>
@@ -12501,7 +12501,7 @@
       <c r="A435" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 22</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B435" s="4" t="n"/>
@@ -12663,7 +12663,7 @@
       <c r="A449" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 18</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B449" s="4" t="n"/>
@@ -12838,7 +12838,7 @@
       <c r="A464" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 19</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B464" s="4" t="n"/>
@@ -13046,7 +13046,7 @@
       <c r="A480" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 16</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B480" s="4" t="n"/>
@@ -13182,7 +13182,7 @@
       <c r="A492" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 11</t>
+Раздел: Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B492" s="4" t="n"/>
@@ -13279,7 +13279,7 @@
       <c r="A501" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 63</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 63</t>
         </is>
       </c>
       <c r="B501" s="4" t="n"/>
@@ -13454,7 +13454,7 @@
       <c r="A516" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Основы ИИ и машинного обучения · УТП: таблица 2, строка 8</t>
+Раздел: Основы ИИ и машинного обучения · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B516" s="4" t="n"/>
@@ -13551,7 +13551,7 @@
       <c r="A525" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 15</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B525" s="4" t="n"/>
@@ -13687,7 +13687,7 @@
       <c r="A537" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 7</t>
+Раздел: Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B537" s="4" t="n"/>
@@ -13784,7 +13784,7 @@
       <c r="A546" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Инфраструктура открытых ключей. · УТП: таблица 2, строка 20</t>
+Раздел: Инфраструктура открытых ключей. · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B546" s="4" t="n"/>
@@ -13881,7 +13881,7 @@
       <c r="A555" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Инфраструктура открытых ключей. · УТП: таблица 2, строка 19</t>
+Раздел: Инфраструктура открытых ключей. · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B555" s="4" t="n"/>
@@ -14043,7 +14043,7 @@
       <c r="A569" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Основы криптографической защиты информации · УТП: таблица 2, строка 8</t>
+Раздел: Основы криптографической защиты информации · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B569" s="4" t="n"/>
@@ -14205,7 +14205,7 @@
       <c r="A583" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B583" s="4" t="n"/>
@@ -14335,7 +14335,7 @@
       <c r="A593" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B593" s="4" t="n"/>
@@ -14465,7 +14465,7 @@
       <c r="A603" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B603" s="4" t="n"/>
@@ -14569,7 +14569,7 @@
       <c r="A611" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B611" s="4" t="n"/>
@@ -14764,7 +14764,7 @@
       <c r="A626" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B626" s="4" t="n"/>
@@ -14868,7 +14868,7 @@
       <c r="A634" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B634" s="4" t="n"/>
@@ -15011,7 +15011,7 @@
       <c r="A645" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B645" s="4" t="n"/>
@@ -15193,7 +15193,7 @@
       <c r="A659" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 6</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B659" s="4" t="n"/>
@@ -15271,7 +15271,7 @@
       <c r="A665" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Нормативное правовое регулирование вопросов кибербезопасности в Республике Беларусь · УТП: таблица 2, строка 7</t>
+Раздел: Нормативное правовое регулирование вопросов кибербезопасности в Республике Беларусь · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B665" s="4" t="n"/>
@@ -15401,7 +15401,7 @@
       <c r="A675" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B675" s="4" t="n"/>
@@ -15505,7 +15505,7 @@
       <c r="A683" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 18</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B683" s="4" t="n"/>
@@ -15609,7 +15609,7 @@
       <c r="A691" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B691" s="4" t="n"/>
@@ -15888,7 +15888,7 @@
       <c r="A714" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Специальное законодательство · УТП: таблица 2, строка 6</t>
+Раздел: Специальное законодательство · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B714" s="4" t="n"/>
@@ -15998,7 +15998,7 @@
       <c r="A724" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Нормативное правовое регулирование вопросов информационной безопасности в Республике Беларусь · УТП: таблица 2, строка 6</t>
+Раздел: Нормативное правовое регулирование вопросов информационной безопасности в Республике Беларусь · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B724" s="4" t="n"/>
@@ -16160,7 +16160,7 @@
       <c r="A738" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Основы ИИ и машинного обучения · УТП: таблица 2, строка 9</t>
+Раздел: Основы ИИ и машинного обучения · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B738" s="4" t="n"/>
@@ -16257,7 +16257,7 @@
       <c r="A747" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 20</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B747" s="4" t="n"/>
@@ -16354,7 +16354,7 @@
       <c r="A756" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 59</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 59</t>
         </is>
       </c>
       <c r="B756" s="4" t="n"/>
@@ -16451,7 +16451,7 @@
       <c r="A765" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Управление информационной безопасностью · УТП: таблица 2, строка 11</t>
+Раздел: Управление информационной безопасностью · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B765" s="4" t="n"/>
@@ -16561,7 +16561,7 @@
       <c r="A775" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Специальное законодательство · УТП: таблица 2, строка 7</t>
+Раздел: Специальное законодательство · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B775" s="4" t="n"/>
@@ -16710,7 +16710,7 @@
       <c r="A788" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 20</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B788" s="4" t="n"/>
@@ -16885,7 +16885,7 @@
       <c r="A803" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 17</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B803" s="4" t="n"/>
@@ -17021,7 +17021,7 @@
       <c r="A815" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 15</t>
+Раздел: Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B815" s="4" t="n"/>
@@ -17118,7 +17118,7 @@
       <c r="A824" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 41</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 41</t>
         </is>
       </c>
       <c r="B824" s="4" t="n"/>
@@ -17280,7 +17280,7 @@
       <c r="A838" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 18</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B838" s="4" t="n"/>
@@ -17377,7 +17377,7 @@
       <c r="A847" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сбор данных и предотвращение атак · УТП: таблица 2, строка 16</t>
+Раздел: Сбор данных и предотвращение атак · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B847" s="4" t="n"/>
@@ -17474,7 +17474,7 @@
       <c r="A856" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 43</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 43</t>
         </is>
       </c>
       <c r="B856" s="4" t="n"/>
@@ -17571,7 +17571,7 @@
       <c r="A865" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 44</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 44</t>
         </is>
       </c>
       <c r="B865" s="4" t="n"/>
@@ -17694,7 +17694,7 @@
       <c r="A876" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Нормативное правовое регулирование вопросов информационной безопасности в Республике Беларусь · УТП: таблица 2, строка 7</t>
+Раздел: Нормативное правовое регулирование вопросов информационной безопасности в Республике Беларусь · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B876" s="4" t="n"/>
@@ -17791,7 +17791,7 @@
       <c r="A885" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Цифровой суверенитет и информационная безопасность · УТП: таблица 2, строка 17</t>
+Раздел: Цифровой суверенитет и информационная безопасность · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B885" s="4" t="n"/>
@@ -17888,7 +17888,7 @@
       <c r="A894" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Инфраструктура открытых ключей. · УТП: таблица 2, строка 18</t>
+Раздел: Инфраструктура открытых ключей. · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B894" s="4" t="n"/>
@@ -17985,7 +17985,7 @@
       <c r="A903" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 10</t>
+Раздел: Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B903" s="4" t="n"/>
@@ -18082,7 +18082,7 @@
       <c r="A912" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 55</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 55</t>
         </is>
       </c>
       <c r="B912" s="4" t="n"/>
@@ -18218,7 +18218,7 @@
       <c r="A924" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 29</t>
+Раздел: Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 29</t>
         </is>
       </c>
       <c r="B924" s="4" t="n"/>
@@ -18315,7 +18315,7 @@
       <c r="A933" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 21</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B933" s="4" t="n"/>
@@ -18412,7 +18412,7 @@
       <c r="A942" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B942" s="4" t="n"/>
@@ -18587,7 +18587,7 @@
       <c r="A957" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Нормативное правовое регулирование вопросов кибербезопасности в Республике Беларусь · УТП: таблица 2, строка 6</t>
+Раздел: Нормативное правовое регулирование вопросов кибербезопасности в Республике Беларусь · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B957" s="4" t="n"/>
@@ -18723,7 +18723,7 @@
       <c r="A969" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B969" s="4" t="n"/>
@@ -18820,7 +18820,7 @@
       <c r="A978" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Введение в кибербезопасность · УТП: таблица 2, строка 11</t>
+Раздел: Введение в кибербезопасность · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B978" s="4" t="n"/>
@@ -18969,7 +18969,7 @@
       <c r="A991" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Проектирование системы защиты информации организации · УТП: таблица 2, строка 13</t>
+Раздел: Проектирование системы защиты информации организации · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B991" s="4" t="n"/>
@@ -19066,7 +19066,7 @@
       <c r="A1000" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Средства криптографической защиты информации · УТП: таблица 2, строка 13</t>
+Раздел: Средства криптографической защиты информации · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B1000" s="4" t="n"/>
@@ -19163,7 +19163,7 @@
       <c r="A1009" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Проектирование системы защиты информации организации · УТП: таблица 2, строка 9</t>
+Раздел: Проектирование системы защиты информации организации · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B1009" s="4" t="n"/>
@@ -19260,7 +19260,7 @@
       <c r="A1018" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 14</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B1018" s="4" t="n"/>
@@ -19357,7 +19357,7 @@
       <c r="A1027" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Нулевая бюрократия и клиентоцентричность · УТП: таблица 2, строка 13</t>
+Раздел: Нулевая бюрократия и клиентоцентричность · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B1027" s="4" t="n"/>
@@ -19454,7 +19454,7 @@
       <c r="A1036" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 19</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B1036" s="4" t="n"/>
@@ -19577,7 +19577,7 @@
       <c r="A1047" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 8</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B1047" s="4" t="n"/>
@@ -19674,7 +19674,7 @@
       <c r="A1056" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Основы криптографической защиты информации · УТП: таблица 2, строка 7</t>
+Раздел: Основы криптографической защиты информации · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1056" s="4" t="n"/>
@@ -19901,7 +19901,7 @@
       <c r="A1075" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Особенности криптографической защиты информации · УТП: таблица 2, строка 17</t>
+Раздел: Особенности криптографической защиты информации · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B1075" s="4" t="n"/>
@@ -19966,7 +19966,7 @@
       <c r="A1080" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B1080" s="4" t="n"/>
@@ -20161,7 +20161,7 @@
       <c r="A1095" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Особенности криптографической защиты информации · УТП: таблица 2, строка 25</t>
+Раздел: Особенности криптографической защиты информации · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B1095" s="4" t="n"/>
@@ -20330,7 +20330,7 @@
       <c r="A1108" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Особенности криптографической защиты информации, обрабатываемой в информационных системах. · УТП: таблица 2, строка 20</t>
+Раздел: Особенности криптографической защиты информации, обрабатываемой в информационных системах. · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B1108" s="4" t="n"/>
@@ -20473,7 +20473,7 @@
       <c r="A1119" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 16</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B1119" s="4" t="n"/>
@@ -20583,7 +20583,7 @@
       <c r="A1129" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Вопросы криптографической защиты информации · УТП: таблица 2, строка 18</t>
+Раздел: Вопросы криптографической защиты информации · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B1129" s="4" t="n"/>
@@ -20797,7 +20797,7 @@
       <c r="A1147" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Криптографическая защита информации · УТП: таблица 2, строка 25</t>
+Раздел: Криптографическая защита информации · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B1147" s="4" t="n"/>
@@ -20862,7 +20862,7 @@
       <c r="A1152" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Особенности криптографической защиты информации · УТП: таблица 2, строка 25</t>
+Раздел: Особенности криптографической защиты информации · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B1152" s="4" t="n"/>
@@ -20998,7 +20998,7 @@
       <c r="A1164" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Основные криптографические алгоритмы и протоколы · УТП: таблица 2, строка 11</t>
+Раздел: Основные криптографические алгоритмы и протоколы · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B1164" s="4" t="n"/>
@@ -21121,7 +21121,7 @@
       <c r="A1175" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Основные криптографические алгоритмы и протоколы · УТП: таблица 2, строка 10</t>
+Раздел: Основные криптографические алгоритмы и протоколы · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B1175" s="4" t="n"/>
@@ -21218,7 +21218,7 @@
       <c r="A1184" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Связь SOAR/TI/SIEM · УТП: таблица 2, строка 68</t>
+Раздел: Связь SOAR/TI/SIEM · УТП: таблица 2, строка 68</t>
         </is>
       </c>
       <c r="B1184" s="4" t="n"/>
@@ -21315,7 +21315,7 @@
       <c r="A1193" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 48</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 48</t>
         </is>
       </c>
       <c r="B1193" s="4" t="n"/>
@@ -21412,7 +21412,7 @@
       <c r="A1202" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 12</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1202" s="4" t="n"/>
@@ -21509,7 +21509,7 @@
       <c r="A1211" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 21</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B1211" s="4" t="n"/>
@@ -21606,7 +21606,7 @@
       <c r="A1220" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Угрозы информационной безопасности · УТП: таблица 2, строка 8</t>
+Раздел: Угрозы информационной безопасности · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B1220" s="4" t="n"/>
@@ -21703,7 +21703,7 @@
       <c r="A1229" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 21</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B1229" s="4" t="n"/>
@@ -21839,7 +21839,7 @@
       <c r="A1241" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Аудит кибербезопасности · УТП: таблица 2, строка 20</t>
+Раздел: Аудит кибербезопасности · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B1241" s="4" t="n"/>
@@ -21936,7 +21936,7 @@
       <c r="A1250" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Управление рисками кибербезопасности · УТП: таблица 2, строка 16</t>
+Раздел: Управление рисками кибербезопасности · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B1250" s="4" t="n"/>
@@ -22033,7 +22033,7 @@
       <c r="A1259" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Угрозы информационной безопасности · УТП: таблица 2, строка 7</t>
+Раздел: Угрозы информационной безопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1259" s="4" t="n"/>
@@ -22130,7 +22130,7 @@
       <c r="A1268" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 17</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B1268" s="4" t="n"/>
@@ -22227,7 +22227,7 @@
       <c r="A1277" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Введение в кибербезопасность · УТП: таблица 2, строка 12</t>
+Раздел: Введение в кибербезопасность · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1277" s="4" t="n"/>
@@ -22324,7 +22324,7 @@
       <c r="A1286" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сбор данных и предотвращение атак · УТП: таблица 2, строка 15</t>
+Раздел: Сбор данных и предотвращение атак · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B1286" s="4" t="n"/>
@@ -22499,7 +22499,7 @@
       <c r="A1301" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Алгоритмы, оценка и объяснимость · УТП: таблица 2, строка 12</t>
+Раздел: Алгоритмы, оценка и объяснимость · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1301" s="4" t="n"/>
@@ -22596,7 +22596,7 @@
       <c r="A1310" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Пилотный проект в сфере цифрового развития как способ реализации цифровой трансформации государственного управления · УТП: таблица 2, строка 25</t>
+Раздел: Пилотный проект в сфере цифрового развития как способ реализации цифровой трансформации государственного управления · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B1310" s="4" t="n"/>
@@ -22693,7 +22693,7 @@
       <c r="A1319" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Управление доступом и аутентификация · УТП: таблица 2, строка 23</t>
+Раздел: Управление доступом и аутентификация · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B1319" s="4" t="n"/>
@@ -22790,7 +22790,7 @@
       <c r="A1328" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 19</t>
+Раздел: Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B1328" s="4" t="n"/>
@@ -22887,7 +22887,7 @@
       <c r="A1337" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 13</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B1337" s="4" t="n"/>
@@ -22984,7 +22984,7 @@
       <c r="A1346" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 17</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B1346" s="4" t="n"/>
@@ -23120,7 +23120,7 @@
       <c r="A1358" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 14</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B1358" s="4" t="n"/>
@@ -23198,7 +23198,7 @@
       <c r="A1364" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1364" s="4" t="n"/>
@@ -23289,7 +23289,7 @@
       <c r="A1371" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 16</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B1371" s="4" t="n"/>
@@ -23380,7 +23380,7 @@
       <c r="A1378" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B1378" s="4" t="n"/>
@@ -23458,7 +23458,7 @@
       <c r="A1384" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 17</t>
+Раздел: Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B1384" s="4" t="n"/>
@@ -23536,7 +23536,7 @@
       <c r="A1390" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 25</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B1390" s="4" t="n"/>
@@ -23737,7 +23737,7 @@
       <c r="A1407" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B1407" s="4" t="n"/>
@@ -23834,7 +23834,7 @@
       <c r="A1416" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 19</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B1416" s="4" t="n"/>
@@ -23957,7 +23957,7 @@
       <c r="A1427" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 23</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B1427" s="4" t="n"/>
@@ -24067,7 +24067,7 @@
       <c r="A1437" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 11</t>
+Раздел: Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B1437" s="4" t="n"/>
@@ -24177,7 +24177,7 @@
       <c r="A1447" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 47</t>
+Раздел: Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 47</t>
         </is>
       </c>
       <c r="B1447" s="4" t="n"/>
@@ -24313,7 +24313,7 @@
       <c r="A1459" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 31</t>
+Раздел: Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 31</t>
         </is>
       </c>
       <c r="B1459" s="4" t="n"/>
@@ -24410,7 +24410,7 @@
       <c r="A1468" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 14</t>
+Раздел: Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B1468" s="4" t="n"/>
@@ -24533,7 +24533,7 @@
       <c r="A1479" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 30</t>
+Раздел: Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 30</t>
         </is>
       </c>
       <c r="B1479" s="4" t="n"/>
@@ -24656,7 +24656,7 @@
       <c r="A1490" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 31</t>
+Раздел: Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 31</t>
         </is>
       </c>
       <c r="B1490" s="4" t="n"/>
@@ -24753,7 +24753,7 @@
       <c r="A1499" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Управление доступом и аутентификация · УТП: таблица 2, строка 26</t>
+Раздел: Управление доступом и аутентификация · УТП: таблица 2, строка 26</t>
         </is>
       </c>
       <c r="B1499" s="4" t="n"/>
@@ -24941,7 +24941,7 @@
       <c r="A1515" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1515" s="4" t="n"/>
@@ -24980,7 +24980,7 @@
       <c r="A1518" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1518" s="4" t="n"/>
@@ -25019,7 +25019,7 @@
       <c r="A1521" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 8</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B1521" s="4" t="n"/>
@@ -25058,7 +25058,7 @@
       <c r="A1524" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1524" s="4" t="n"/>
@@ -25097,7 +25097,7 @@
       <c r="A1527" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 19</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B1527" s="4" t="n"/>
@@ -25136,7 +25136,7 @@
       <c r="A1530" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1530" s="4" t="n"/>
@@ -25240,7 +25240,7 @@
       <c r="A1538" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1538" s="4" t="n"/>
@@ -25279,7 +25279,7 @@
       <c r="A1541" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1541" s="4" t="n"/>
@@ -25319,7 +25319,7 @@
       <c r="A1544" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1544" s="4" t="n"/>
@@ -25514,7 +25514,7 @@
       <c r="A1559" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
+Раздел: Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1559" s="4" t="n"/>
@@ -25657,7 +25657,7 @@
       <c r="A1570" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 7</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности. · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1570" s="4" t="n"/>
@@ -25755,7 +25755,7 @@
       <c r="A1579" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 8</t>
+Раздел: Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B1579" s="4" t="n"/>
@@ -25852,7 +25852,7 @@
       <c r="A1588" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 38</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 38</t>
         </is>
       </c>
       <c r="B1588" s="4" t="n"/>
@@ -25962,7 +25962,7 @@
       <c r="A1598" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Раздел VI Системы управления информационной безопасностью и событиями безопасности (SIEM). · Тема добавлена непосредственно из обновлённой программы</t>
+Раздел: VI Системы управления информационной безопасностью и событиями безопасности (SIEM). · Тема добавлена непосредственно из обновлённой программы</t>
         </is>
       </c>
       <c r="B1598" s="4" t="n"/>
@@ -26059,7 +26059,7 @@
       <c r="A1607" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Нулевая бюрократия и клиентоцентричность · УТП: таблица 2, строка 12</t>
+Раздел: Нулевая бюрократия и клиентоцентричность · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1607" s="4" t="n"/>
@@ -26273,7 +26273,7 @@
       <c r="A1625" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 14</t>
+Раздел: Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B1625" s="4" t="n"/>
@@ -26370,7 +26370,7 @@
       <c r="A1634" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 23</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B1634" s="4" t="n"/>
@@ -26545,7 +26545,7 @@
       <c r="A1649" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 18</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B1649" s="4" t="n"/>
@@ -26779,7 +26779,7 @@
       <c r="A1667" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 15</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B1667" s="4" t="n"/>
@@ -26876,7 +26876,7 @@
       <c r="A1676" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Управление доступом и аутентификация · УТП: таблица 2, строка 25</t>
+Раздел: Управление доступом и аутентификация · УТП: таблица 2, строка 25</t>
         </is>
       </c>
       <c r="B1676" s="4" t="n"/>
@@ -26973,7 +26973,7 @@
       <c r="A1685" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 51</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 51</t>
         </is>
       </c>
       <c r="B1685" s="4" t="n"/>
@@ -27070,7 +27070,7 @@
       <c r="A1694" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 36</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 36</t>
         </is>
       </c>
       <c r="B1694" s="4" t="n"/>
@@ -27219,7 +27219,7 @@
       <c r="A1707" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Основы ИИ и машинного обучения · УТП: таблица 2, строка 7</t>
+Раздел: Основы ИИ и машинного обучения · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B1707" s="4" t="n"/>
@@ -27316,7 +27316,7 @@
       <c r="A1716" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 14</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B1716" s="4" t="n"/>
@@ -27413,7 +27413,7 @@
       <c r="A1725" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Угрозы информационной безопасности · УТП: таблица 2, строка 6</t>
+Раздел: Угрозы информационной безопасности · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B1725" s="4" t="n"/>
@@ -27575,7 +27575,7 @@
       <c r="A1739" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 21</t>
+Раздел: Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B1739" s="4" t="n"/>
@@ -27737,7 +27737,7 @@
       <c r="A1753" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 20</t>
+Раздел: Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B1753" s="4" t="n"/>
@@ -27886,7 +27886,7 @@
       <c r="A1766" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 19</t>
+Раздел: Практические кейсы применения ИИ в ИБ · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B1766" s="4" t="n"/>
@@ -28035,7 +28035,7 @@
       <c r="A1779" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Проектирование системы защиты информации организации · УТП: таблица 2, строка 12</t>
+Раздел: Проектирование системы защиты информации организации · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1779" s="4" t="n"/>
@@ -28210,7 +28210,7 @@
       <c r="A1794" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Алгоритмы, оценка и объяснимость · УТП: таблица 2, строка 13</t>
+Раздел: Алгоритмы, оценка и объяснимость · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B1794" s="4" t="n"/>
@@ -28307,7 +28307,7 @@
       <c r="A1803" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 34</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 34</t>
         </is>
       </c>
       <c r="B1803" s="4" t="n"/>
@@ -28443,7 +28443,7 @@
       <c r="A1815" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 27</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 27</t>
         </is>
       </c>
       <c r="B1815" s="4" t="n"/>
@@ -28540,7 +28540,7 @@
       <c r="A1824" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 8</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B1824" s="4" t="n"/>
@@ -28767,7 +28767,7 @@
       <c r="A1843" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 10</t>
+Раздел: Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B1843" s="4" t="n"/>
@@ -28890,7 +28890,7 @@
       <c r="A1854" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Особенности криптографической защиты информации · УТП: таблица 2, строка 18</t>
+Раздел: Особенности криптографической защиты информации · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B1854" s="4" t="n"/>
@@ -28929,7 +28929,7 @@
       <c r="A1857" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Особенности криптографической защиты информации · УТП: таблица 2, строка 26</t>
+Раздел: Особенности криптографической защиты информации · УТП: таблица 2, строка 26</t>
         </is>
       </c>
       <c r="B1857" s="4" t="n"/>
@@ -28994,7 +28994,7 @@
       <c r="A1862" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Особенности криптографической защиты информации, обрабатываемой в информационных системах. · УТП: таблица 2, строка 21</t>
+Раздел: Особенности криптографической защиты информации, обрабатываемой в информационных системах. · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B1862" s="4" t="n"/>
@@ -29169,7 +29169,7 @@
       <c r="A1877" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Алгоритмы, оценка и объяснимость · УТП: таблица 2, строка 11</t>
+Раздел: Алгоритмы, оценка и объяснимость · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B1877" s="4" t="n"/>
@@ -29266,7 +29266,7 @@
       <c r="A1886" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Средства криптографической защиты информации · УТП: таблица 2, строка 15</t>
+Раздел: Средства криптографической защиты информации · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B1886" s="4" t="n"/>
@@ -29363,7 +29363,7 @@
       <c r="A1895" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 40</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 40</t>
         </is>
       </c>
       <c r="B1895" s="4" t="n"/>
@@ -29486,7 +29486,7 @@
       <c r="A1906" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Средства криптографической защиты информации · УТП: таблица 2, строка 14</t>
+Раздел: Средства криптографической защиты информации · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B1906" s="4" t="n"/>
@@ -29635,7 +29635,7 @@
       <c r="A1919" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Оценка эффективности защищенности инфраструктуры. Реагирование на киберинциденты · УТП: таблица 2, строка 21</t>
+Раздел: Оценка эффективности защищенности инфраструктуры. Реагирование на киберинциденты · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B1919" s="4" t="n"/>
@@ -29758,7 +29758,7 @@
       <c r="A1930" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 21</t>
+Раздел: Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B1930" s="4" t="n"/>
@@ -29855,7 +29855,7 @@
       <c r="A1939" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 35</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 35</t>
         </is>
       </c>
       <c r="B1939" s="4" t="n"/>
@@ -29965,7 +29965,7 @@
       <c r="A1949" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Основы защиты персональных данных. Законодательство о персональных данных. · УТП: таблица 2, строка 9</t>
+Раздел: Основы защиты персональных данных. Законодательство о персональных данных. · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B1949" s="4" t="n"/>
@@ -30063,7 +30063,7 @@
       <c r="A1958" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Введение в кибербезопасность · УТП: таблица 2, строка 10</t>
+Раздел: Введение в кибербезопасность · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B1958" s="4" t="n"/>
@@ -30160,7 +30160,7 @@
       <c r="A1967" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Управление информационной безопасностью · УТП: таблица 2, строка 12</t>
+Раздел: Управление информационной безопасностью · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B1967" s="4" t="n"/>
@@ -30296,7 +30296,7 @@
       <c r="A1979" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Подтверждение соответствия средств защиты информации · УТП: таблица 2, строка 9</t>
+Раздел: Подтверждение соответствия средств защиты информации · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B1979" s="4" t="n"/>
@@ -30406,7 +30406,7 @@
       <c r="A1989" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Особенности эксплуатации системы защиты информации организации · УТП: таблица 2, строка 34</t>
+Раздел: Особенности эксплуатации системы защиты информации организации · УТП: таблица 2, строка 34</t>
         </is>
       </c>
       <c r="B1989" s="4" t="n"/>
@@ -30503,7 +30503,7 @@
       <c r="A1998" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 20</t>
+Раздел: Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B1998" s="4" t="n"/>
@@ -30613,7 +30613,7 @@
       <c r="A2008" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Оценка эффективности защищенности инфраструктуры. Реагирование на киберинциденты · УТП: таблица 2, строка 19</t>
+Раздел: Оценка эффективности защищенности инфраструктуры. Реагирование на киберинциденты · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B2008" s="4" t="n"/>
@@ -30749,7 +30749,7 @@
       <c r="A2020" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Аудит кибербезопасности · УТП: таблица 2, строка 21</t>
+Раздел: Аудит кибербезопасности · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B2020" s="4" t="n"/>
@@ -30846,7 +30846,7 @@
       <c r="A2029" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 9</t>
+Раздел: Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2029" s="4" t="n"/>
@@ -30943,7 +30943,7 @@
       <c r="A2038" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 46</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 46</t>
         </is>
       </c>
       <c r="B2038" s="4" t="n"/>
@@ -31040,7 +31040,7 @@
       <c r="A2047" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 62</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 62</t>
         </is>
       </c>
       <c r="B2047" s="4" t="n"/>
@@ -31176,7 +31176,7 @@
       <c r="A2059" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 28</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 28</t>
         </is>
       </c>
       <c r="B2059" s="4" t="n"/>
@@ -31273,7 +31273,7 @@
       <c r="A2068" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 52</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 52</t>
         </is>
       </c>
       <c r="B2068" s="4" t="n"/>
@@ -31422,7 +31422,7 @@
       <c r="A2081" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 33</t>
+Раздел: Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 33</t>
         </is>
       </c>
       <c r="B2081" s="4" t="n"/>
@@ -31532,7 +31532,7 @@
       <c r="A2091" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Раздел VI Системы управления информационной безопасностью и событиями безопасности (SIEM). · Тема добавлена непосредственно из обновлённой программы</t>
+Раздел: VI Системы управления информационной безопасностью и событиями безопасности (SIEM). · Тема добавлена непосредственно из обновлённой программы</t>
         </is>
       </c>
       <c r="B2091" s="4" t="n"/>
@@ -31642,7 +31642,7 @@
       <c r="A2101" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 17</t>
+Раздел: Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2101" s="4" t="n"/>
@@ -31739,7 +31739,7 @@
       <c r="A2110" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 27</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 27</t>
         </is>
       </c>
       <c r="B2110" s="4" t="n"/>
@@ -31875,7 +31875,7 @@
       <c r="A2122" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Аудит кибербезопасности · УТП: таблица 2, строка 19</t>
+Раздел: Аудит кибербезопасности · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B2122" s="4" t="n"/>
@@ -31972,7 +31972,7 @@
       <c r="A2131" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Пилотный проект в сфере цифрового развития как способ реализации цифровой трансформации государственного управления · УТП: таблица 2, строка 24</t>
+Раздел: Пилотный проект в сфере цифрового развития как способ реализации цифровой трансформации государственного управления · УТП: таблица 2, строка 24</t>
         </is>
       </c>
       <c r="B2131" s="4" t="n"/>
@@ -32108,7 +32108,7 @@
       <c r="A2143" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 32</t>
+Раздел: Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 32</t>
         </is>
       </c>
       <c r="B2143" s="4" t="n"/>
@@ -32205,7 +32205,7 @@
       <c r="A2152" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Управление информационной безопасностью · УТП: таблица 2, строка 13</t>
+Раздел: Управление информационной безопасностью · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B2152" s="4" t="n"/>
@@ -32315,7 +32315,7 @@
       <c r="A2162" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B2162" s="4" t="n"/>
@@ -32354,7 +32354,7 @@
       <c r="A2165" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B2165" s="4" t="n"/>
@@ -32451,7 +32451,7 @@
       <c r="A2174" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Практический блок · УТП: таблица 2, строка 28</t>
+Раздел: Практический блок · УТП: таблица 2, строка 28</t>
         </is>
       </c>
       <c r="B2174" s="4" t="n"/>
@@ -32548,7 +32548,7 @@
       <c r="A2183" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 18</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B2183" s="4" t="n"/>
@@ -32645,7 +32645,7 @@
       <c r="A2192" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 17</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2192" s="4" t="n"/>
@@ -32755,7 +32755,7 @@
       <c r="A2202" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 23</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B2202" s="4" t="n"/>
@@ -32930,7 +32930,7 @@
       <c r="A2217" s="3" t="inlineStr">
         <is>
           <t>ПТИИМ — Применение технологий искусственного интеллекта и машинного обучения в информационной и кибербезопасности
-Применение ИИ в ИБ · УТП: таблица 2, строка 15</t>
+Раздел: Применение ИИ в ИБ · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B2217" s="4" t="n"/>
@@ -33027,7 +33027,7 @@
       <c r="A2226" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сбор данных и предотвращение атак · УТП: таблица 2, строка 17</t>
+Раздел: Сбор данных и предотвращение атак · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2226" s="4" t="n"/>
@@ -33215,7 +33215,7 @@
       <c r="A2242" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Управление рисками кибербезопасности · УТП: таблица 2, строка 17</t>
+Раздел: Управление рисками кибербезопасности · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2242" s="4" t="n"/>
@@ -33312,7 +33312,7 @@
       <c r="A2251" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в киберкриминалистику · УТП: таблица 2, строка 26</t>
+Раздел: Введение в киберкриминалистику · УТП: таблица 2, строка 26</t>
         </is>
       </c>
       <c r="B2251" s="4" t="n"/>
@@ -33435,7 +33435,7 @@
       <c r="A2262" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 22</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B2262" s="4" t="n"/>
@@ -33500,7 +33500,7 @@
       <c r="A2267" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 21</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B2267" s="4" t="n"/>
@@ -33597,7 +33597,7 @@
       <c r="A2276" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 6</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B2276" s="4" t="n"/>
@@ -33694,7 +33694,7 @@
       <c r="A2285" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 19</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 19</t>
         </is>
       </c>
       <c r="B2285" s="4" t="n"/>
@@ -33791,7 +33791,7 @@
       <c r="A2294" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 22</t>
+Раздел: Управление цифровой трансформацией: офисы цифровизации · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B2294" s="4" t="n"/>
@@ -33888,7 +33888,7 @@
       <c r="A2303" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Методологические основы обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 10</t>
+Раздел: Методологические основы обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B2303" s="4" t="n"/>
@@ -33985,7 +33985,7 @@
       <c r="A2312" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 18</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B2312" s="4" t="n"/>
@@ -34082,7 +34082,7 @@
       <c r="A2321" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 64</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 64</t>
         </is>
       </c>
       <c r="B2321" s="4" t="n"/>
@@ -34179,7 +34179,7 @@
       <c r="A2330" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Угрозы информационной безопасности · УТП: таблица 2, строка 9</t>
+Раздел: Угрозы информационной безопасности · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2330" s="4" t="n"/>
@@ -34341,7 +34341,7 @@
       <c r="A2344" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 12</t>
+Раздел: Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B2344" s="4" t="n"/>
@@ -34490,7 +34490,7 @@
       <c r="A2357" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Проектирование системы защиты информации организации · УТП: таблица 2, строка 14</t>
+Раздел: Проектирование системы защиты информации организации · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B2357" s="4" t="n"/>
@@ -34587,7 +34587,7 @@
       <c r="A2366" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Практический блок · УТП: таблица 2, строка 27</t>
+Раздел: Практический блок · УТП: таблица 2, строка 27</t>
         </is>
       </c>
       <c r="B2366" s="4" t="n"/>
@@ -34710,7 +34710,7 @@
       <c r="A2377" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Аттестация системы защиты информации организации · УТП: таблица 2, строка 31</t>
+Раздел: Аттестация системы защиты информации организации · УТП: таблица 2, строка 31</t>
         </is>
       </c>
       <c r="B2377" s="4" t="n"/>
@@ -34846,7 +34846,7 @@
       <c r="A2389" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 26</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 26</t>
         </is>
       </c>
       <c r="B2389" s="4" t="n"/>
@@ -34995,7 +34995,7 @@
       <c r="A2402" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Проектирование системы защиты информации организации · УТП: таблица 2, строка 15</t>
+Раздел: Проектирование системы защиты информации организации · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B2402" s="4" t="n"/>
@@ -35092,7 +35092,7 @@
       <c r="A2411" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 14</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B2411" s="4" t="n"/>
@@ -35131,7 +35131,7 @@
       <c r="A2414" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 17</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2414" s="4" t="n"/>
@@ -35254,7 +35254,7 @@
       <c r="A2425" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Аттестация системы защиты информации организации · УТП: таблица 2, строка 32</t>
+Раздел: Аттестация системы защиты информации организации · УТП: таблица 2, строка 32</t>
         </is>
       </c>
       <c r="B2425" s="4" t="n"/>
@@ -35390,7 +35390,7 @@
       <c r="A2437" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 17</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2437" s="4" t="n"/>
@@ -35507,7 +35507,7 @@
       <c r="A2446" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 16</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B2446" s="4" t="n"/>
@@ -35572,7 +35572,7 @@
       <c r="A2451" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 18</t>
+Раздел: Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B2451" s="4" t="n"/>
@@ -35760,7 +35760,7 @@
       <c r="A2467" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Оценка эффективности защищенности инфраструктуры. Реагирование на киберинциденты · УТП: таблица 2, строка 20</t>
+Раздел: Оценка эффективности защищенности инфраструктуры. Реагирование на киберинциденты · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B2467" s="4" t="n"/>
@@ -35857,7 +35857,7 @@
       <c r="A2476" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 61</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 61</t>
         </is>
       </c>
       <c r="B2476" s="4" t="n"/>
@@ -35954,7 +35954,7 @@
       <c r="A2485" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 15</t>
+Раздел: Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B2485" s="4" t="n"/>
@@ -36051,7 +36051,7 @@
       <c r="A2494" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 37</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 37</t>
         </is>
       </c>
       <c r="B2494" s="4" t="n"/>
@@ -36200,7 +36200,7 @@
       <c r="A2507" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2507" s="4" t="n"/>
@@ -36323,7 +36323,7 @@
       <c r="A2518" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B2518" s="4" t="n"/>
@@ -36459,7 +36459,7 @@
       <c r="A2530" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2530" s="4" t="n"/>
@@ -36569,7 +36569,7 @@
       <c r="A2540" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 44</t>
+Раздел: Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 44</t>
         </is>
       </c>
       <c r="B2540" s="4" t="n"/>
@@ -36634,7 +36634,7 @@
       <c r="A2545" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 49</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 49</t>
         </is>
       </c>
       <c r="B2545" s="4" t="n"/>
@@ -36731,7 +36731,7 @@
       <c r="A2554" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 53</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 53</t>
         </is>
       </c>
       <c r="B2554" s="4" t="n"/>
@@ -36828,7 +36828,7 @@
       <c r="A2563" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 54</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 54</t>
         </is>
       </c>
       <c r="B2563" s="4" t="n"/>
@@ -36925,7 +36925,7 @@
       <c r="A2572" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 9</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2572" s="4" t="n"/>
@@ -37022,7 +37022,7 @@
       <c r="A2581" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 11</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B2581" s="4" t="n"/>
@@ -37119,7 +37119,7 @@
       <c r="A2590" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Связь SOAR/TI/SIEM · УТП: таблица 2, строка 70</t>
+Раздел: Связь SOAR/TI/SIEM · УТП: таблица 2, строка 70</t>
         </is>
       </c>
       <c r="B2590" s="4" t="n"/>
@@ -37463,7 +37463,7 @@
       <c r="A2618" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 15</t>
+Раздел: Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B2618" s="4" t="n"/>
@@ -37625,7 +37625,7 @@
       <c r="A2632" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Методологические основы обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 9</t>
+Раздел: Методологические основы обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2632" s="4" t="n"/>
@@ -37722,7 +37722,7 @@
       <c r="A2641" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 24</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 24</t>
         </is>
       </c>
       <c r="B2641" s="4" t="n"/>
@@ -37819,7 +37819,7 @@
       <c r="A2650" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 16</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B2650" s="4" t="n"/>
@@ -37929,7 +37929,7 @@
       <c r="A2660" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Раздел VII SOAR, TIP – автоматизация реагирования. · Тема добавлена непосредственно из обновлённой программы</t>
+Раздел: VII SOAR, TIP – автоматизация реагирования. · Тема добавлена непосредственно из обновлённой программы</t>
         </is>
       </c>
       <c r="B2660" s="4" t="n"/>
@@ -38026,7 +38026,7 @@
       <c r="A2669" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Связь SOAR/TI/SIEM · УТП: таблица 2, строка 67</t>
+Раздел: Связь SOAR/TI/SIEM · УТП: таблица 2, строка 67</t>
         </is>
       </c>
       <c r="B2669" s="4" t="n"/>
@@ -38123,7 +38123,7 @@
       <c r="A2678" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Автоматизация обработки инцидентов · УТП: таблица 2, строка 65</t>
+Раздел: Автоматизация обработки инцидентов · УТП: таблица 2, строка 65</t>
         </is>
       </c>
       <c r="B2678" s="4" t="n"/>
@@ -38220,7 +38220,7 @@
       <c r="A2687" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 32</t>
+Раздел: Сканирование уязвимостей, скрипты реагирования, скрипты для сбора логов · УТП: таблица 2, строка 32</t>
         </is>
       </c>
       <c r="B2687" s="4" t="n"/>
@@ -38330,7 +38330,7 @@
       <c r="A2697" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 45</t>
+Раздел: Отработка практических заданий на базе киберполигона · УТП: таблица 2, строка 45</t>
         </is>
       </c>
       <c r="B2697" s="4" t="n"/>
@@ -38395,7 +38395,7 @@
       <c r="A2702" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 57</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 57</t>
         </is>
       </c>
       <c r="B2702" s="4" t="n"/>
@@ -38492,7 +38492,7 @@
       <c r="A2711" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Защита конечных устройств · УТП: таблица 2, строка 42</t>
+Раздел: Защита конечных устройств · УТП: таблица 2, строка 42</t>
         </is>
       </c>
       <c r="B2711" s="4" t="n"/>
@@ -38589,7 +38589,7 @@
       <c r="A2720" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 20</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B2720" s="4" t="n"/>
@@ -38686,7 +38686,7 @@
       <c r="A2729" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Защита конечных устройств · УТП: таблица 2, строка 39</t>
+Раздел: Защита конечных устройств · УТП: таблица 2, строка 39</t>
         </is>
       </c>
       <c r="B2729" s="4" t="n"/>
@@ -38835,7 +38835,7 @@
       <c r="A2742" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Криптографическая защита информации · УТП: таблица 2, строка 26</t>
+Раздел: Криптографическая защита информации · УТП: таблица 2, строка 26</t>
         </is>
       </c>
       <c r="B2742" s="4" t="n"/>
@@ -38913,7 +38913,7 @@
       <c r="A2748" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Криптографическая защита информации. · УТП: таблица 2, строка 23</t>
+Раздел: Криптографическая защита информации. · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B2748" s="4" t="n"/>
@@ -38978,7 +38978,7 @@
       <c r="A2753" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B2753" s="4" t="n"/>
@@ -39043,7 +39043,7 @@
       <c r="A2758" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 24</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 24</t>
         </is>
       </c>
       <c r="B2758" s="4" t="n"/>
@@ -39166,7 +39166,7 @@
       <c r="A2769" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B2769" s="4" t="n"/>
@@ -39244,7 +39244,7 @@
       <c r="A2775" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B2775" s="4" t="n"/>
@@ -39283,7 +39283,7 @@
       <c r="A2778" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 10</t>
+Раздел: Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B2778" s="4" t="n"/>
@@ -39322,7 +39322,7 @@
       <c r="A2781" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 23</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B2781" s="4" t="n"/>
@@ -39426,7 +39426,7 @@
       <c r="A2789" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 21</t>
+Раздел: Технические меры по обеспечению кибербезопасности · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B2789" s="4" t="n"/>
@@ -39523,7 +39523,7 @@
       <c r="A2798" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 56</t>
+Раздел: Интеграция и использование TI в ЦКБ · УТП: таблица 2, строка 56</t>
         </is>
       </c>
       <c r="B2798" s="4" t="n"/>
@@ -39620,7 +39620,7 @@
       <c r="A2807" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B2807" s="4" t="n"/>
@@ -39769,7 +39769,7 @@
       <c r="A2820" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 16</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B2820" s="4" t="n"/>
@@ -39905,7 +39905,7 @@
       <c r="A2832" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 18</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B2832" s="4" t="n"/>
@@ -40002,7 +40002,7 @@
       <c r="A2841" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 17</t>
+Раздел: Маршрутизация. IPv4 и IPv6 адресация · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B2841" s="4" t="n"/>
@@ -40125,7 +40125,7 @@
       <c r="A2852" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Криптографическая защита информации · УТП: таблица 2, строка 27</t>
+Раздел: Криптографическая защита информации · УТП: таблица 2, строка 27</t>
         </is>
       </c>
       <c r="B2852" s="4" t="n"/>
@@ -40222,7 +40222,7 @@
       <c r="A2861" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Защита конечных устройств · УТП: таблица 2, строка 41</t>
+Раздел: Защита конечных устройств · УТП: таблица 2, строка 41</t>
         </is>
       </c>
       <c r="B2861" s="4" t="n"/>
@@ -40319,7 +40319,7 @@
       <c r="A2870" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 47</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 47</t>
         </is>
       </c>
       <c r="B2870" s="4" t="n"/>
@@ -40416,7 +40416,7 @@
       <c r="A2879" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 45</t>
+Раздел: Интеграция и использование SOAR в ЦКБ · УТП: таблица 2, строка 45</t>
         </is>
       </c>
       <c r="B2879" s="4" t="n"/>
@@ -40513,7 +40513,7 @@
       <c r="A2888" s="3" t="inlineStr">
         <is>
           <t>РКИОК — Реагирование на киберинциденты и отражение кибератак
-Введение в SOAR и TI · УТП: таблица 2, строка 39</t>
+Раздел: Введение в SOAR и TI · УТП: таблица 2, строка 39</t>
         </is>
       </c>
       <c r="B2888" s="4" t="n"/>
@@ -40623,7 +40623,7 @@
       <c r="A2898" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 30</t>
+Раздел: Системы управления информационной безопасностью и событиями безопасности (SIEM) · УТП: таблица 2, строка 30</t>
         </is>
       </c>
       <c r="B2898" s="4" t="n"/>
@@ -40720,7 +40720,7 @@
       <c r="A2907" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 22</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B2907" s="4" t="n"/>
@@ -40830,7 +40830,7 @@
       <c r="A2917" s="3" t="inlineStr">
         <is>
           <t>КЗИ — Криптографическая защита информации
-Средства криптографической защиты информации · УТП: таблица 2, строка 16</t>
+Раздел: Средства криптографической защиты информации · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B2917" s="4" t="n"/>
@@ -41122,7 +41122,7 @@
       <c r="A2941" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B2941" s="4" t="n"/>
@@ -41356,7 +41356,7 @@
       <c r="A2959" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 9</t>
+Раздел: Проектирование, создание и аттестация систем защиты информации. · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B2959" s="4" t="n"/>
@@ -41713,7 +41713,7 @@
       <c r="A2988" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 22</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 22</t>
         </is>
       </c>
       <c r="B2988" s="4" t="n"/>
@@ -41849,7 +41849,7 @@
       <c r="A3000" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Проектирование системы защиты информации организации · УТП: таблица 2, строка 10</t>
+Раздел: Проектирование системы защиты информации организации · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B3000" s="4" t="n"/>
@@ -42128,7 +42128,7 @@
       <c r="A3023" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 14</t>
+Раздел: Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B3023" s="4" t="n"/>
@@ -42472,7 +42472,7 @@
       <c r="A3051" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B3051" s="4" t="n"/>
@@ -42823,7 +42823,7 @@
       <c r="A3078" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B3078" s="4" t="n"/>
@@ -43226,7 +43226,7 @@
       <c r="A3109" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B3109" s="4" t="n"/>
@@ -43304,7 +43304,7 @@
       <c r="A3115" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 13</t>
+Раздел: Практические аспекты обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B3115" s="4" t="n"/>
@@ -43707,7 +43707,7 @@
       <c r="A3146" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 14</t>
+Раздел: Практические аспекты обеспечения кибербезопасности · УТП: таблица 2, строка 14</t>
         </is>
       </c>
       <c r="B3146" s="4" t="n"/>
@@ -43804,7 +43804,7 @@
       <c r="A3155" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Нормативное правовое регулирование вопросов кибербезопасности в Республике Беларусь · УТП: таблица 2, строка 8</t>
+Раздел: Нормативное правовое регулирование вопросов кибербезопасности в Республике Беларусь · УТП: таблица 2, строка 8</t>
         </is>
       </c>
       <c r="B3155" s="4" t="n"/>
@@ -43901,7 +43901,7 @@
       <c r="A3164" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Тренды киберпреступности. Кибератаки с использованием методов социальной инженерии. · УТП: таблица 2, строка 11</t>
+Раздел: Тренды киберпреступности. Кибератаки с использованием методов социальной инженерии. · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B3164" s="4" t="n"/>
@@ -44258,7 +44258,7 @@
       <c r="A3193" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Управление киберинцидентами · УТП: таблица 2, строка 20</t>
+Раздел: Управление киберинцидентами · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B3193" s="4" t="n"/>
@@ -44492,7 +44492,7 @@
       <c r="A3211" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Управление киберинцидентами · УТП: таблица 2, строка 23</t>
+Раздел: Управление киберинцидентами · УТП: таблица 2, строка 23</t>
         </is>
       </c>
       <c r="B3211" s="4" t="n"/>
@@ -44589,7 +44589,7 @@
       <c r="A3220" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Защита конечных устройств · УТП: таблица 2, строка 40</t>
+Раздел: Защита конечных устройств · УТП: таблица 2, строка 40</t>
         </is>
       </c>
       <c r="B3220" s="4" t="n"/>
@@ -44686,7 +44686,7 @@
       <c r="A3229" s="3" t="inlineStr">
         <is>
           <t>АКБ — Администратор кибербезопасности
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B3229" s="4" t="n"/>
@@ -44725,7 +44725,7 @@
       <c r="A3232" s="3" t="inlineStr">
         <is>
           <t>БКТ — Безопасность компьютерных технологий
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 12</t>
         </is>
       </c>
       <c r="B3232" s="4" t="n"/>
@@ -44764,7 +44764,7 @@
       <c r="A3235" s="3" t="inlineStr">
         <is>
           <t>ТЗПД — Техническая защита персональных данных
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 11</t>
         </is>
       </c>
       <c r="B3235" s="4" t="n"/>
@@ -44803,7 +44803,7 @@
       <c r="A3238" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Методологические основы обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 9</t>
+Раздел: Методологические основы обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B3238" s="4" t="n"/>
@@ -44900,7 +44900,7 @@
       <c r="A3247" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 18</t>
+Раздел: Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 18</t>
         </is>
       </c>
       <c r="B3247" s="4" t="n"/>
@@ -44978,7 +44978,7 @@
       <c r="A3253" s="3" t="inlineStr">
         <is>
           <t>ККС — Кибербезопасность корпоративных систем
-Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 13</t>
+Раздел: Правовые и организационные меры по обеспечению кибербезопасности · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B3253" s="4" t="n"/>
@@ -45043,7 +45043,7 @@
       <c r="A3258" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 13</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B3258" s="4" t="n"/>
@@ -45082,7 +45082,7 @@
       <c r="A3261" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 13</t>
         </is>
       </c>
       <c r="B3261" s="4" t="n"/>
@@ -45121,7 +45121,7 @@
       <c r="A3264" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 20</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B3264" s="4" t="n"/>
@@ -45218,7 +45218,7 @@
       <c r="A3273" s="3" t="inlineStr">
         <is>
           <t>ЗИОЗ — Защита информационной инфраструктуры организаций здравоохранения
-Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
+Раздел: Методологические основы обеспечения кибербезопасности · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B3273" s="4" t="n"/>
@@ -45445,7 +45445,7 @@
       <c r="A3292" s="3" t="inlineStr">
         <is>
           <t>АУРИК — Аудит, управление рисками и инцидентами кибербезопасности
-Управление рисками кибербезопасности · УТП: таблица 2, строка 15</t>
+Раздел: Управление рисками кибербезопасности · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B3292" s="4" t="n"/>
@@ -45594,7 +45594,7 @@
       <c r="A3305" s="3" t="inlineStr">
         <is>
           <t>КВОИ — Кибербезопасность критически важных объектов информатизации
-Методологические основы обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 10</t>
+Раздел: Методологические основы обеспечения кибербезопасности критически важных объектов информатизации · УТП: таблица 2, строка 10</t>
         </is>
       </c>
       <c r="B3305" s="4" t="n"/>
@@ -45691,7 +45691,7 @@
       <c r="A3314" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 16</t>
+Раздел: Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B3314" s="4" t="n"/>
@@ -45788,7 +45788,7 @@
       <c r="A3323" s="3" t="inlineStr">
         <is>
           <t>ПСАЭ — Проектирование, создание, аттестация и эксплуатация систем защиты информации
-Настройка системы защиты информации организации · УТП: таблица 2, строка 20</t>
+Раздел: Настройка системы защиты информации организации · УТП: таблица 2, строка 20</t>
         </is>
       </c>
       <c r="B3323" s="4" t="n"/>
@@ -45885,7 +45885,7 @@
       <c r="A3332" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 15</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B3332" s="4" t="n"/>
@@ -45982,7 +45982,7 @@
       <c r="A3341" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 16</t>
+Раздел: Практические аспекты обеспечения кибербезопасности корпоративных систем · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B3341" s="4" t="n"/>
@@ -46079,7 +46079,7 @@
       <c r="A3350" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы обеспечения кибербезопасности · УТП: таблица 2, строка 21</t>
+Раздел: Основы обеспечения кибербезопасности · УТП: таблица 2, строка 21</t>
         </is>
       </c>
       <c r="B3350" s="4" t="n"/>
@@ -46176,7 +46176,7 @@
       <c r="A3359" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 15</t>
+Раздел: Меры по обеспечению кибербезопасности. · УТП: таблица 2, строка 15</t>
         </is>
       </c>
       <c r="B3359" s="4" t="n"/>
@@ -46241,7 +46241,7 @@
       <c r="A3364" s="3" t="inlineStr">
         <is>
           <t>ОКМ — Основы обеспечения кибербезопасности. маршрутизация. IPv4- и IPv6-адресация
-Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
+Раздел: Основы обеспечения кибербезопасности. Законодательство в области обеспечения кибербезопасности · УТП: таблица 2, строка 9</t>
         </is>
       </c>
       <c r="B3364" s="4" t="n"/>
@@ -46338,7 +46338,7 @@
       <c r="A3373" s="3" t="inlineStr">
         <is>
           <t>ОПКС — Основы построения компьютерных сетей и обеспечения кибербезопасности
-Основы построения компьютерных сетей · УТП: таблица 2, строка 7</t>
+Раздел: Основы построения компьютерных сетей · УТП: таблица 2, строка 7</t>
         </is>
       </c>
       <c r="B3373" s="4" t="n"/>
@@ -46435,7 +46435,7 @@
       <c r="A3382" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-SOAR, TIP, XDR- Автоматизация реагирования · УТП: таблица 2, строка 35</t>
+Раздел: SOAR, TIP, XDR- Автоматизация реагирования · УТП: таблица 2, строка 35</t>
         </is>
       </c>
       <c r="B3382" s="4" t="n"/>
@@ -46532,7 +46532,7 @@
       <c r="A3391" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-SOAR, TIP, XDR- Автоматизация реагирования · УТП: таблица 2, строка 36</t>
+Раздел: SOAR, TIP, XDR- Автоматизация реагирования · УТП: таблица 2, строка 36</t>
         </is>
       </c>
       <c r="B3391" s="4" t="n"/>
@@ -46642,7 +46642,7 @@
       <c r="A3401" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-SOAR, TIP, XDR- Автоматизация реагирования · УТП: таблица 2, строка 37</t>
+Раздел: SOAR, TIP, XDR- Автоматизация реагирования · УТП: таблица 2, строка 37</t>
         </is>
       </c>
       <c r="B3401" s="4" t="n"/>
@@ -46739,7 +46739,7 @@
       <c r="A3410" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 6</t>
+Раздел: Стратегия государства: экономика данных и цифровое государство (2026–2030) · УТП: таблица 2, строка 6</t>
         </is>
       </c>
       <c r="B3410" s="4" t="n"/>
@@ -46836,7 +46836,7 @@
       <c r="A3419" s="3" t="inlineStr">
         <is>
           <t>ЦТГУ — Цифровая трансформация государственного управления
-Цифровой суверенитет и информационная безопасность · УТП: таблица 2, строка 16</t>
+Раздел: Цифровой суверенитет и информационная безопасность · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B3419" s="4" t="n"/>
@@ -46985,7 +46985,7 @@
       <c r="A3432" s="3" t="inlineStr">
         <is>
           <t>ЗИКС — Защита информации в корпоративных системах
-Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 16</t>
+Раздел: Обеспечение функционирования системы защиты информации в процессе эксплуатации информационной системы. · УТП: таблица 2, строка 16</t>
         </is>
       </c>
       <c r="B3432" s="4" t="n"/>
@@ -47082,7 +47082,7 @@
       <c r="A3441" s="3" t="inlineStr">
         <is>
           <t>ТК — Технологии кибербезопасности: от spoofing-атак до VPN и межсетевых экранов
-Особенности криптографической защиты информации · УТП: таблица 2, строка 26</t>
+Раздел: Особенности криптографической защиты информации · УТП: таблица 2, строка 26</t>
         </is>
       </c>
       <c r="B3441" s="4" t="n"/>
@@ -47179,7 +47179,7 @@
       <c r="A3450" s="3" t="inlineStr">
         <is>
           <t>КО — Кибербезопасность государственных и иных организаций
-Криптографическая защита информации. · УТП: таблица 2, строка 24</t>
+Раздел: Криптографическая защита информации. · УТП: таблица 2, строка 24</t>
         </is>
       </c>
       <c r="B3450" s="4" t="n"/>
@@ -47276,7 +47276,7 @@
       <c r="A3459" s="3" t="inlineStr">
         <is>
           <t>ОКБО — Обеспечение кибербезопасности организаций
-Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 17</t>
+Раздел: Основные функции центров обеспечения кибербезопасности и реагирования на киберинциденты объектов информационной инфраструктуры государственных органов и иных организаций (ЦКБ), процессы информационной безопасности · УТП: таблица 2, строка 17</t>
         </is>
       </c>
       <c r="B3459" s="4" t="n"/>

</xml_diff>